<commit_message>
modified worksheet with files generator for both ab and vm
</commit_message>
<xml_diff>
--- a/vm/Division General Method  Flag M.xlsx
+++ b/vm/Division General Method  Flag M.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\abacus-worksheet\vm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{642D9DC5-B253-4CD9-8A9D-CB00D22DC00E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0AC0CDD-78F8-43E8-97F2-8774860E6FDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{10B0DCFA-4AF4-4F82-BFCF-291A17A868C6}"/>
   </bookViews>

</xml_diff>